<commit_message>
added references for new service accounts
</commit_message>
<xml_diff>
--- a/diagrams/Naming Convention Reference.xlsx
+++ b/diagrams/Naming Convention Reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Code Repositories\personal\Home Lab\lab_infra\diagrams\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\lab_infra\diagrams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985A61C6-16A3-47A3-9F27-98806A8973B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D183324-E6D1-4D08-8484-13C1DD9347BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22944" yWindow="0" windowWidth="23232" windowHeight="25296" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="2628" windowWidth="34560" windowHeight="18600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subsystems" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
   <si>
     <t>Subsystem Name</t>
   </si>
@@ -63,6 +63,69 @@
   </si>
   <si>
     <t>rodc</t>
+  </si>
+  <si>
+    <t>ansible</t>
+  </si>
+  <si>
+    <t>an</t>
+  </si>
+  <si>
+    <t>join</t>
+  </si>
+  <si>
+    <t>Domain Joins</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>Domain Account for Ansible to use to join machines to the domain</t>
+  </si>
+  <si>
+    <t>DHCP</t>
+  </si>
+  <si>
+    <t>DHCP Server</t>
+  </si>
+  <si>
+    <t>dhcp</t>
+  </si>
+  <si>
+    <t>Network Stack</t>
+  </si>
+  <si>
+    <t>ns</t>
+  </si>
+  <si>
+    <t>Access Switch</t>
+  </si>
+  <si>
+    <t>ac</t>
+  </si>
+  <si>
+    <t>Distro Switch</t>
+  </si>
+  <si>
+    <t>di</t>
+  </si>
+  <si>
+    <t>East-West Firewall</t>
+  </si>
+  <si>
+    <t>ewfw</t>
+  </si>
+  <si>
+    <t>North-South Firewall</t>
+  </si>
+  <si>
+    <t>nsfw</t>
+  </si>
+  <si>
+    <t>RODC Admin</t>
+  </si>
+  <si>
+    <t>RODC Server Admin Account to use when accessing RODCs</t>
   </si>
 </sst>
 </file>
@@ -380,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81598938-9837-42A1-86CC-8227B9B21A2B}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -403,6 +466,22 @@
         <v>7</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -410,7 +489,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -461,6 +540,76 @@
         <v>11</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -468,7 +617,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD2B409-1E54-4972-B66B-652E6A5AF996}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -477,7 +626,7 @@
     <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -489,6 +638,43 @@
       </c>
       <c r="D1" t="s">
         <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates and typo fixes for dhcp
</commit_message>
<xml_diff>
--- a/diagrams/Naming Convention Reference.xlsx
+++ b/diagrams/Naming Convention Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\lab_infra\diagrams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D183324-E6D1-4D08-8484-13C1DD9347BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CB0C47-DB1B-429A-B31A-2EF0E7465045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="2628" windowWidth="34560" windowHeight="18600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="2628" windowWidth="34560" windowHeight="18600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subsystems" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
   <si>
     <t>Subsystem Name</t>
   </si>
@@ -126,6 +126,12 @@
   </si>
   <si>
     <t>RODC Server Admin Account to use when accessing RODCs</t>
+  </si>
+  <si>
+    <t>GUI Workstation</t>
+  </si>
+  <si>
+    <t>work</t>
   </si>
 </sst>
 </file>
@@ -489,7 +495,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -608,6 +614,20 @@
       </c>
       <c r="D8" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates for gitlab install
</commit_message>
<xml_diff>
--- a/diagrams/Naming Convention Reference.xlsx
+++ b/diagrams/Naming Convention Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\lab_infra\diagrams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CB0C47-DB1B-429A-B31A-2EF0E7465045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1CB1B52-7240-44E7-BC28-CD6DC02B5E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="2628" windowWidth="34560" windowHeight="18600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="2628" windowWidth="34560" windowHeight="18600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subsystems" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="42">
   <si>
     <t>Subsystem Name</t>
   </si>
@@ -132,6 +132,27 @@
   </si>
   <si>
     <t>work</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>co</t>
+  </si>
+  <si>
+    <t>glab</t>
+  </si>
+  <si>
+    <t>GitLab</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>GitLab LDAP Bind</t>
+  </si>
+  <si>
+    <t>Service Accounts to allow GitLab to bind to LDAP</t>
   </si>
 </sst>
 </file>
@@ -449,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81598938-9837-42A1-86CC-8227B9B21A2B}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -488,6 +509,14 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -495,7 +524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -630,6 +659,20 @@
         <v>34</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -637,13 +680,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD2B409-1E54-4972-B66B-652E6A5AF996}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -697,6 +741,23 @@
         <v>32</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>